<commit_message>
Actualizar Efevoo con la propuesta formal Marca Blanca Agregador
Toma los términos de la propuesta formal del 25-sep-2026: recurrencia
desde producción, marcas desde 2027, costo 3DS para tarjeta no presente,
sin mínimo por transacciones y sin reparto de MDR.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NRbY4gaPNszaKyKvPy5v1Z
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Sofo_Plus_PagaTodo_vs_Efevoo_5A.xlsx
+++ b/modelos/Modelo_Sofo_Plus_PagaTodo_vs_Efevoo_5A.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="259">
   <si>
     <t xml:space="preserve">Comité de Nuevos Productos — Cobranza Cupón con TPV | Banco PagaTodo vs Efevoo Pay</t>
   </si>
@@ -64,7 +64,10 @@
     <t xml:space="preserve">% del margen neto MDR que se queda el proveedor</t>
   </si>
   <si>
-    <t xml:space="preserve">Costo por transacción (USD)</t>
+    <t xml:space="preserve">Costo por transacción tarjeta presente (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por transacción no presente con 3DS (USD)</t>
   </si>
   <si>
     <t xml:space="preserve">Registro anual ante marcas (USD/año, desde el año 2)</t>
@@ -145,7 +148,7 @@
     <t xml:space="preserve">Margen neto MDR mínimo con Efevoo para empatar con PagaTodo</t>
   </si>
   <si>
-    <t xml:space="preserve">Si la "Tasa agregador" de Efevoo deja a Sofo Plus un margen neto menor a este %, conviene PagaTodo.</t>
+    <t xml:space="preserve">Si después de intercambio, marcas y adquirente a Sofo Plus le queda un margen neto menor a este %, conviene PagaTodo.</t>
   </si>
   <si>
     <t xml:space="preserve">4. Supuestos del caso base (editar en la hoja Supuestos)</t>
@@ -196,10 +199,10 @@
     <t xml:space="preserve">3. PagaTodo: la tabla de mínimos de la propuesta tiene un error ("Mes 1 y 2 / Mes 2 y 3 / Mes 5+"); se usan los tramos 1-2, 3-4 y 5+.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Efevoo: se asume que Sofo Plus retiene el 100% del margen neto MDR. Falta confirmar qué es la "Tasa agregador" 2.06% / 1.45% / 2.95% y quién absorbe intercambio y Prosa.</t>
+    <t xml:space="preserve">4. Efevoo (propuesta formal): no cobra % sobre volumen ni reparte MDR; Sofo Plus retiene el margen neto. Validar el costo del adquirente en el esquema multi-adquirente.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Efevoo: la propuesta menciona un mínimo de volumen por transacciones sin monto; capturarlo en Supuestos cuando se confirme.</t>
+    <t xml:space="preserve">5. Efevoo: la propuesta formal no fija mínimo por transacciones y no incluye terminales; el precio de TPV (USD 131) viene de la presentación comercial.</t>
   </si>
   <si>
     <t xml:space="preserve">6. Efevoo: operar como agregador implica costos propios (cumplimiento, contracargos, soporte, liquidación) que no están en la propuesta. Ver la holgura en el indicador de la fila 43.</t>
@@ -382,58 +385,76 @@
     <t xml:space="preserve">  Umbral de TPV activas para el segundo pago</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Efevoo Pay — Agregador marca blanca, propuesta 25-sep-2026 (USD)</t>
+    <t xml:space="preserve">5. Efevoo Pay — Propuesta formal Marca Blanca Agregador, 25-sep-2026 (USD)</t>
   </si>
   <si>
     <t xml:space="preserve">Implementación inicial (USD, pago único)</t>
   </si>
   <si>
-    <t xml:space="preserve">Efevoo pág. 29. Incluye el registro ante Visa/MC del primer año.</t>
+    <t xml:space="preserve">Propuesta formal Efevoo: USD 20,000 pago único. Incluye el registro ante Visa/MasterCard del primer año.</t>
   </si>
   <si>
     <t xml:space="preserve">Renta dashboard de control interno y clientes (USD/mes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Efevoo pág. 30.</t>
+    <t xml:space="preserve">Desglose de la presentación comercial (pág. 30). La propuesta formal confirma recurrencia total de USD 3,950/mes.</t>
   </si>
   <si>
     <t xml:space="preserve">Renta fija switch transaccional Alpha Connect (USD/mes)</t>
   </si>
   <si>
+    <t xml:space="preserve">Efevoo pág. 30.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Servidores dedicados (USD/mes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total cuota fija mensual (USD)</t>
+    <t xml:space="preserve">Total recurrencia mensual (USD) — se cobra desde que la solución entra a producción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta formal: USD 3,950/mes. El mes 1 del plan se considera el arranque en producción.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo por transacción con tarjeta presente (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Efevoo pág. 30-31.</t>
+    <t xml:space="preserve">Propuesta formal Efevoo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por transacción con tarjeta no presente con 3DS (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta formal Efevoo. Solo aplica a e-commerce / links de pago.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de transacciones con tarjeta no presente (e-commerce)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobranza cupón con TPV = tarjeta presente, por eso 0%. Subirlo si se cobra también con links de pago.</t>
   </si>
   <si>
     <t xml:space="preserve">Mínimo mensual por transacciones (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">La propuesta dice que hay "un mínimo de volumen fijo mensual" pero no da el monto. Capturar cuando lo confirmen.</t>
+    <t xml:space="preserve">La propuesta formal no establece mínimo mensual (la presentación lo mencionaba sin monto).</t>
   </si>
   <si>
     <t xml:space="preserve">Registro anual ante las marcas Visa/MC (USD/año)</t>
   </si>
   <si>
-    <t xml:space="preserve">Efevoo pág. 31-32. El primer año está incluido en la implementación.</t>
+    <t xml:space="preserve">Propuesta formal: USD 10,000 anuales a partir del segundo año (2027), cobro al año vencido.</t>
   </si>
   <si>
     <t xml:space="preserve">  Mes del primer cobro anual de marcas</t>
   </si>
   <si>
-    <t xml:space="preserve">La propuesta dice "al año vencido, finales de 2027". Se asume mes 13 del plan; después se repite cada 12 meses.</t>
+    <t xml:space="preserve">Propuesta formal: al año vencido. Se asume mes 13 del plan (primer aniversario); después cada 12 meses.</t>
   </si>
   <si>
     <t xml:space="preserve">Precio de compra por TPV (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Efevoo pág. 32: Ultra con impresora USD 131; Smart sin impresora USD 112. Sin IVA.</t>
+    <t xml:space="preserve">No viene en la propuesta formal. Precio de la presentación comercial (pág. 32): Ultra USD 131; Smart USD 112. Sin IVA. Confirmar.</t>
   </si>
   <si>
     <t xml:space="preserve">¿Se reutilizan las TPV de créditos liquidados? (1 = Sí, 0 = No)</t>
@@ -445,7 +466,7 @@
     <t xml:space="preserve">Margen neto MDR para Sofo Plus con Efevoo (% de facturación)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supone que Sofo Plus retiene el 100% del margen neto (no hay split). CONFIRMAR qué significa la "Tasa agregador" 2.06% / 1.45% / 2.95% de Efevoo (pág. 20).</t>
+    <t xml:space="preserve">La propuesta formal NO cobra % sobre volumen ni reparte MDR: Sofo Plus retiene el margen neto (MDR al comercio menos intercambio, marcas y adquirente). Validar el costo del adquirente en el esquema multi-adquirente.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo operativo propio de operar como agregador (MXN/mes)</t>
@@ -2179,11 +2200,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="19043884"/>
-        <c:axId val="57607045"/>
+        <c:axId val="62217035"/>
+        <c:axId val="78923771"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="19043884"/>
+        <c:axId val="62217035"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2249,7 +2270,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57607045"/>
+        <c:crossAx val="78923771"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2257,7 +2278,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57607045"/>
+        <c:axId val="78923771"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2333,7 +2354,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19043884"/>
+        <c:crossAx val="62217035"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2644,11 +2665,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="95869336"/>
-        <c:axId val="8149497"/>
+        <c:axId val="56326802"/>
+        <c:axId val="80190238"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95869336"/>
+        <c:axId val="56326802"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2680,7 +2701,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8149497"/>
+        <c:crossAx val="80190238"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2688,7 +2709,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8149497"/>
+        <c:axId val="80190238"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2730,7 +2751,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95869336"/>
+        <c:crossAx val="56326802"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3234,8 +3255,8 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="str">
-        <f aca="false">"Tipo de cambio "&amp;TEXT(Supuestos!$C$7,"0.00")&amp;" MXN/USD · Propuestas: PagaTodo 17-sep-2026 y Efevoo 25-sep-2026 (vigencia 30 días)"</f>
-        <v>Tipo de cambio 17.00 MXN/USD · Propuestas: PagaTodo 17-sep-2026 y Efevoo 25-sep-2026 (vigencia 30 días)</v>
+        <f aca="false">"Tipo de cambio "&amp;TEXT(Supuestos!$C$7,"0.00")&amp;" MXN/USD · Propuestas: PagaTodo 17-sep-2026 y Efevoo propuesta formal Marca Blanca Agregador 25-sep-2026"</f>
+        <v>Tipo de cambio 17.00 MXN/USD · Propuestas: PagaTodo 17-sep-2026 y Efevoo propuesta formal Marca Blanca Agregador 25-sep-2026</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -3718,7 +3739,7 @@
         <v>5000</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">Supuestos!$C$52</f>
+        <f aca="false">Supuestos!$C$54</f>
         <v>0</v>
       </c>
       <c r="E11" s="1"/>
@@ -3790,7 +3811,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">Supuestos!$C$55</f>
+        <f aca="false">Supuestos!$C$57</f>
         <v>131</v>
       </c>
       <c r="E12" s="1"/>
@@ -3933,7 +3954,7 @@
         <v>0.5</v>
       </c>
       <c r="D14" s="12" t="n">
-        <f aca="false">IF(Supuestos!$C$20=0,0,1-Supuestos!$C$57/Supuestos!$C$20)</f>
+        <f aca="false">IF(Supuestos!$C$20=0,0,1-Supuestos!$C$59/Supuestos!$C$20)</f>
         <v>0</v>
       </c>
       <c r="E14" s="1"/>
@@ -4071,12 +4092,12 @@
       <c r="B16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <f aca="false">Supuestos!$C$53</f>
-        <v>10000</v>
+      <c r="C16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <f aca="false">Supuestos!$C$52</f>
+        <v>0.18</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -4139,9 +4160,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
+      <c r="B17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <f aca="false">Supuestos!$C$55</f>
+        <v>10000</v>
+      </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -4204,7 +4232,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
@@ -4270,7 +4298,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C19" s="17" t="n">
         <v>1</v>
@@ -4288,7 +4316,7 @@
         <v>5</v>
       </c>
       <c r="H19" s="16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -4348,7 +4376,7 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -4414,7 +4442,7 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">SUMIF('BP PagaTodo'!$C$6:$BJ$6,C$19,'BP PagaTodo'!$C$15:$BJ$15)</f>
@@ -4498,7 +4526,7 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C22" s="19" t="n">
         <f aca="false">SUMIF('BP PagaTodo'!$C$6:$BJ$6,C$19,'BP PagaTodo'!$C$18:$BJ$18)</f>
@@ -4582,7 +4610,7 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C23" s="19" t="n">
         <f aca="false">SUMIF('BP PagaTodo'!$C$6:$BJ$6,C$19,'BP PagaTodo'!$C$23:$BJ$23)-C22</f>
@@ -4666,7 +4694,7 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="21" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C24" s="22" t="n">
         <f aca="false">SUMIF('BP PagaTodo'!$C$6:$BJ$6,C$19,'BP PagaTodo'!$C$25:$BJ$25)</f>
@@ -4750,7 +4778,7 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -4816,7 +4844,7 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
       <c r="B26" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C26" s="19" t="n">
         <f aca="false">SUMIF('BP Efevoo'!$C$6:$BJ$6,C$19,'BP Efevoo'!$C$15:$BJ$15)</f>
@@ -4900,7 +4928,7 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C27" s="19" t="n">
         <f aca="false">SUMIF('BP Efevoo'!$C$6:$BJ$6,C$19,'BP Efevoo'!$C$18:$BJ$18)</f>
@@ -4984,7 +5012,7 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
       <c r="B28" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C28" s="19" t="n">
         <f aca="false">SUMIF('BP Efevoo'!$C$6:$BJ$6,C$19,'BP Efevoo'!$C$25:$BJ$25)-C27</f>
@@ -5068,7 +5096,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1"/>
       <c r="B29" s="21" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C29" s="22" t="n">
         <f aca="false">SUMIF('BP Efevoo'!$C$6:$BJ$6,C$19,'BP Efevoo'!$C$27:$BJ$27)</f>
@@ -5152,7 +5180,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1"/>
       <c r="B30" s="23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C30" s="24" t="n">
         <f aca="false">C29-C24</f>
@@ -5300,7 +5328,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>4</v>
@@ -5370,7 +5398,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1"/>
       <c r="B33" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C33" s="19" t="n">
         <f aca="false">NPV(((1+Supuestos!$C$8)^(1/12)-1),'BP PagaTodo'!C25:BJ25)</f>
@@ -5442,7 +5470,7 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1"/>
       <c r="B34" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C34" s="25" t="n">
         <f aca="false">'BP PagaTodo'!BJ26</f>
@@ -5514,7 +5542,7 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1"/>
       <c r="B35" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C35" s="19" t="n">
         <f aca="false">SUM('BP PagaTodo'!C31:BJ31)</f>
@@ -5586,7 +5614,7 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1"/>
       <c r="B36" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C36" s="19" t="n">
         <f aca="false">IF(MIN('BP PagaTodo'!C32:BJ32)=999,"no se alcanza",MIN('BP PagaTodo'!C32:BJ32))</f>
@@ -5658,7 +5686,7 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1"/>
       <c r="B37" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C37" s="19" t="n">
         <f aca="false">MIN('BP PagaTodo'!C25:BJ25)</f>
@@ -5730,7 +5758,7 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1"/>
       <c r="B38" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C38" s="19" t="n">
         <f aca="false">COUNTIF('BP PagaTodo'!C25:BJ25,"&lt;0")</f>
@@ -5802,7 +5830,7 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1"/>
       <c r="B39" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C39" s="12" t="n">
         <f aca="false">IF(H21=0,0,H24/H21)</f>
@@ -5874,7 +5902,7 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1"/>
       <c r="B40" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C40" s="25" t="n">
         <f aca="false">'Economía por Crédito'!C22</f>
@@ -5946,7 +5974,7 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1"/>
       <c r="B41" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C41" s="25" t="n">
         <f aca="false">'BP PagaTodo'!BJ25</f>
@@ -6018,7 +6046,7 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1"/>
       <c r="B42" s="23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C42" s="26" t="n">
         <f aca="false">'Economía por Crédito'!C24</f>
@@ -6087,14 +6115,14 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1"/>
       <c r="B43" s="23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C43" s="24" t="n">
         <f aca="false">H30/60</f>
         <v>1166980.82247592</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -6158,14 +6186,14 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1"/>
       <c r="B44" s="23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C44" s="27" t="n">
-        <f aca="false">Supuestos!$C$57-IF(SUM('Cartera 60M'!C76:BJ76)=0,0,H30/SUM('Cartera 60M'!C76:BJ76))</f>
+        <f aca="false">Supuestos!$C$59-IF(SUM('Cartera 60M'!C76:BJ76)=0,0,H30/SUM('Cartera 60M'!C76:BJ76))</f>
         <v>0.00297673362052872</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -6229,7 +6257,7 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1"/>
       <c r="B45" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C45" s="15"/>
       <c r="D45" s="15"/>
@@ -6295,7 +6323,7 @@
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1"/>
       <c r="B46" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C46" s="25" t="n">
         <f aca="false">Supuestos!$C$11</f>
@@ -6364,7 +6392,7 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1"/>
       <c r="B47" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C47" s="25" t="n">
         <f aca="false">Supuestos!$C$13</f>
@@ -6433,7 +6461,7 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1"/>
       <c r="B48" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C48" s="7" t="str">
         <f aca="false">TEXT(Supuestos!$C$14,"0.0%")&amp;" / "&amp;Supuestos!$C$15&amp;" meses"</f>
@@ -6502,7 +6530,7 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1"/>
       <c r="B49" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C49" s="10" t="n">
         <f aca="false">Supuestos!$C$16</f>
@@ -6571,7 +6599,7 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1"/>
       <c r="B50" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C50" s="10" t="n">
         <f aca="false">Supuestos!$C$20</f>
@@ -6640,7 +6668,7 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1"/>
       <c r="B51" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C51" s="25" t="n">
         <f aca="false">Supuestos!$C$19</f>
@@ -6709,7 +6737,7 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1"/>
       <c r="B52" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C52" s="7" t="str">
         <f aca="false">TEXT(Supuestos!$C$24,"$#,##0")&amp;" / mes "&amp;Supuestos!$C$25</f>
@@ -6778,7 +6806,7 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1"/>
       <c r="B53" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C53" s="25" t="n">
         <f aca="false">'Cartera 60M'!BJ75</f>
@@ -6847,7 +6875,7 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1"/>
       <c r="B54" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C54" s="25" t="n">
         <f aca="false">'Cartera 60M'!BJ66</f>
@@ -6916,10 +6944,10 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1"/>
       <c r="B55" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C55" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="D55" s="1"/>
@@ -6985,7 +7013,7 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1"/>
       <c r="B56" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C56" s="10" t="n">
         <f aca="false">Supuestos!$C$8</f>
@@ -7118,7 +7146,7 @@
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1"/>
       <c r="B58" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C58" s="15"/>
       <c r="D58" s="15"/>
@@ -7184,7 +7212,7 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1"/>
       <c r="B59" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
@@ -7250,7 +7278,7 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1"/>
       <c r="B60" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
@@ -7316,7 +7344,7 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1"/>
       <c r="B61" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -7382,7 +7410,7 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1"/>
       <c r="B62" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
@@ -7448,7 +7476,7 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1"/>
       <c r="B63" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
@@ -7514,7 +7542,7 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1"/>
       <c r="B64" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
@@ -7580,7 +7608,7 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1"/>
       <c r="B65" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
@@ -7646,7 +7674,7 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1"/>
       <c r="B66" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
@@ -7840,7 +7868,7 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1"/>
       <c r="B69" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C69" s="15"/>
       <c r="D69" s="15"/>
@@ -7906,7 +7934,7 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1"/>
       <c r="B70" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C70" s="25" t="n">
         <f aca="false">'BP PagaTodo'!C5</f>
@@ -8658,7 +8686,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -8677,7 +8705,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -8686,7 +8714,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -8709,42 +8737,42 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>17</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C8" s="29" t="n">
         <v>0.15</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8757,48 +8785,48 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" s="30" t="n">
         <v>1000000</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" s="31" t="n">
         <v>1.5</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" s="19" t="n">
         <f aca="false">Supuestos!$C$11*Supuestos!$C$12</f>
@@ -8810,92 +8838,92 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C14" s="11" t="n">
         <v>0.33</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C15" s="30" t="n">
         <v>12</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
       <c r="B16" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" s="11" t="n">
         <v>0.1158</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C17" s="11" t="n">
         <v>0.03</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C18" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C19" s="32" t="n">
         <v>500</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C20" s="11" t="n">
         <v>0.006</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8908,81 +8936,81 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C23" s="30" t="n">
         <v>2</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C24" s="30" t="n">
         <v>500000000</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C25" s="30" t="n">
         <v>48</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
       <c r="B26" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C27" s="34" t="n">
         <v>1.5</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8995,22 +9023,22 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1"/>
       <c r="B29" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1"/>
       <c r="B30" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>10</v>
@@ -9020,13 +9048,13 @@
         <v>170</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1"/>
       <c r="B31" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>15</v>
@@ -9036,52 +9064,52 @@
         <v>255</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C32" s="30" t="n">
         <v>7</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1"/>
       <c r="B33" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C33" s="11" t="n">
         <v>0.5</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1"/>
       <c r="B34" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C34" s="11" t="n">
         <v>0.0075</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1"/>
       <c r="B35" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>0</v>
@@ -9091,26 +9119,26 @@
         <v>0</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1"/>
       <c r="B36" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C36" s="32" t="n">
         <v>2</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1"/>
       <c r="B37" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C37" s="9" t="n">
         <v>2500</v>
@@ -9120,26 +9148,26 @@
         <v>42500</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1"/>
       <c r="B38" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C38" s="32" t="n">
         <v>4</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1"/>
       <c r="B39" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C39" s="9" t="n">
         <v>5000</v>
@@ -9149,13 +9177,13 @@
         <v>85000</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1"/>
       <c r="B40" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C40" s="9" t="n">
         <v>15000</v>
@@ -9165,46 +9193,46 @@
         <v>255000</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1"/>
       <c r="B41" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C41" s="11" t="n">
         <v>0.5</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1"/>
       <c r="B42" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C42" s="30" t="n">
         <v>6</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1"/>
       <c r="B43" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C43" s="30" t="n">
         <v>20</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9217,22 +9245,22 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1"/>
       <c r="B45" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1"/>
       <c r="B46" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C46" s="9" t="n">
         <v>20000</v>
@@ -9242,13 +9270,13 @@
         <v>340000</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1"/>
       <c r="B47" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C47" s="9" t="n">
         <v>3000</v>
@@ -9258,13 +9286,13 @@
         <v>51000</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1"/>
       <c r="B48" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C48" s="9" t="n">
         <v>750</v>
@@ -9274,13 +9302,13 @@
         <v>12750</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1"/>
       <c r="B49" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>200</v>
@@ -9290,13 +9318,13 @@
         <v>3400</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1"/>
       <c r="B50" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C50" s="35" t="n">
         <f aca="false">Supuestos!$C$47+Supuestos!$C$48+Supuestos!$C$49</f>
@@ -9306,12 +9334,14 @@
         <f aca="false">C50*Supuestos!$C$7</f>
         <v>67150</v>
       </c>
-      <c r="E50" s="1"/>
+      <c r="E50" s="3" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1"/>
       <c r="B51" s="7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>0.03</v>
@@ -9321,107 +9351,136 @@
         <v>0.51</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1"/>
       <c r="B52" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="C52" s="36" t="n">
-        <v>0</v>
+        <v>131</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>0.18</v>
       </c>
       <c r="D52" s="25" t="n">
         <f aca="false">C52*Supuestos!$C$7</f>
-        <v>0</v>
+        <v>3.06</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1"/>
       <c r="B53" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="C53" s="9" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D53" s="25" t="n">
-        <f aca="false">C53*Supuestos!$C$7</f>
-        <v>170000</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="1"/>
       <c r="E53" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1"/>
       <c r="B54" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="C54" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="D54" s="1"/>
+        <v>135</v>
+      </c>
+      <c r="C54" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="25" t="n">
+        <f aca="false">C54*Supuestos!$C$7</f>
+        <v>0</v>
+      </c>
       <c r="E54" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1"/>
       <c r="B55" s="7" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C55" s="9" t="n">
-        <v>131</v>
+        <v>10000</v>
       </c>
       <c r="D55" s="25" t="n">
         <f aca="false">C55*Supuestos!$C$7</f>
-        <v>2227</v>
+        <v>170000</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1"/>
       <c r="B56" s="7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C56" s="32" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D56" s="1"/>
       <c r="E56" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1"/>
       <c r="B57" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C57" s="29" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="D57" s="1"/>
+        <v>141</v>
+      </c>
+      <c r="C57" s="36" t="n">
+        <v>131</v>
+      </c>
+      <c r="D57" s="25" t="n">
+        <f aca="false">C57*Supuestos!$C$7</f>
+        <v>2227</v>
+      </c>
       <c r="E57" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1"/>
       <c r="B58" s="7" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C58" s="32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1"/>
+      <c r="B59" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C59" s="29" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="D59" s="1"/>
+      <c r="E59" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1"/>
+      <c r="B60" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C60" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="1"/>
+      <c r="E60" s="3" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -9466,7 +9525,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -9486,7 +9545,7 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="7" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C4" s="25" t="n">
         <f aca="false">Supuestos!$C$13</f>
@@ -9500,7 +9559,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="7" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">Supuestos!$C$14</f>
@@ -9514,7 +9573,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="7" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C6" s="37" t="n">
         <f aca="false">C5/12</f>
@@ -9528,7 +9587,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="7" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">Supuestos!$C$15</f>
@@ -9542,7 +9601,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="7" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">C4*C6/(1-(1+C6)^(-C7))</f>
@@ -9556,7 +9615,7 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="7" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">C4*Supuestos!$C$17</f>
@@ -9570,7 +9629,7 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="7" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">C4*Supuestos!$C$16/12</f>
@@ -9593,22 +9652,22 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="16" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10627,7 +10686,7 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1"/>
       <c r="B52" s="16" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C52" s="38"/>
       <c r="D52" s="1"/>
@@ -10638,7 +10697,7 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1"/>
       <c r="B53" s="7" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C53" s="19" t="n">
         <f aca="false">SUM(E14:E49)</f>
@@ -10652,7 +10711,7 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1"/>
       <c r="B54" s="7" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C54" s="19" t="n">
         <f aca="false">C9</f>
@@ -10666,7 +10725,7 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1"/>
       <c r="B55" s="7" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C55" s="19" t="n">
         <f aca="false">C53+C54</f>
@@ -10680,7 +10739,7 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1"/>
       <c r="B56" s="7" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C56" s="19" t="n">
         <f aca="false">SUM(C14:C49)*Supuestos!$C$16/12</f>
@@ -10694,7 +10753,7 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1"/>
       <c r="B57" s="23" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C57" s="20" t="n">
         <f aca="false">C55-C56</f>
@@ -10796,7 +10855,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -10862,7 +10921,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -10992,7 +11051,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="25" t="n">
         <f aca="false">Supuestos!$C$13</f>
@@ -11061,7 +11120,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="7" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C6" s="37" t="n">
         <f aca="false">Supuestos!$C$14/12</f>
@@ -11130,7 +11189,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="7" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">Supuestos!$C$15</f>
@@ -11199,7 +11258,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="7" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">C5*C6/(1-(1+C6)^(-C7))</f>
@@ -11268,7 +11327,7 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="7" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">Supuestos!$C$23</f>
@@ -11337,7 +11396,7 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C10" s="25" t="n">
         <f aca="false">Supuestos!$C$24</f>
@@ -11406,7 +11465,7 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="7" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C11" s="25" t="n">
         <f aca="false">Supuestos!$C$25</f>
@@ -11475,7 +11534,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="7" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C12" s="39" t="n">
         <f aca="false">SUM(C24:C59)</f>
@@ -11544,7 +11603,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="7" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C13" s="39" t="n">
         <f aca="false">SUMPRODUCT(D24:D59,C24:C59)</f>
@@ -11613,7 +11672,7 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="7" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C14" s="40" t="n">
         <f aca="false">IF(C13=0,0,(C10/C5-C9*C12)/C13)</f>
@@ -11682,7 +11741,7 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="7" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C15" s="41" t="str">
         <f aca="false">Supuestos!$C$26</f>
@@ -11751,7 +11810,7 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
       <c r="B16" s="7" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C16" s="42" t="n">
         <f aca="false">Supuestos!$C$27</f>
@@ -11820,7 +11879,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="7" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C17" s="40" t="n">
         <f aca="false">IF(C15="Rampa manual",C16,C14)</f>
@@ -11889,7 +11948,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="7" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">MIN(Supuestos!$C$42,MIN(C80:BJ80))</f>
@@ -11958,7 +12017,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="7" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C19" s="19" t="n">
         <f aca="false">INDEX(C75:BJ75,1,C11)</f>
@@ -12027,7 +12086,7 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="7" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">IF(C10=0,0,C19/C10)</f>
@@ -12224,13 +12283,13 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="16" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -14950,7 +15009,7 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1"/>
       <c r="B61" s="6" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C61" s="15"/>
       <c r="D61" s="15"/>
@@ -15016,7 +15075,7 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1"/>
       <c r="B62" s="23" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C62" s="43" t="n">
         <v>1</v>
@@ -15261,7 +15320,7 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1"/>
       <c r="B63" s="7" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C63" s="19" t="n">
         <f aca="false">ROUNDUP(C62/12,0)</f>
@@ -15507,7 +15566,7 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1"/>
       <c r="B64" s="7" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C64" s="19" t="n">
         <f aca="false">ROUND(MAX(0,$C$9+(MIN(C62,$C$11)-1)*$C$17),0)</f>
@@ -15753,7 +15812,7 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1"/>
       <c r="B65" s="7" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C65" s="19" t="n">
         <f aca="false">C64</f>
@@ -15999,7 +16058,7 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1"/>
       <c r="B66" s="7" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C66" s="19" t="n">
         <f aca="false">C65-IF(C62&gt;$C$7,INDEX($C$65:$BJ$65,1,C62-$C$7),0)</f>
@@ -16245,7 +16304,7 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1"/>
       <c r="B67" s="7" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C67" s="25" t="n">
         <f aca="false">C66*Supuestos!$C$18</f>
@@ -16491,7 +16550,7 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1"/>
       <c r="B68" s="7" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C68" s="19" t="n">
         <f aca="false">MAX(0,IF(C62-Supuestos!$C$32+1&gt;=1,INDEX($C$65:$BJ$65,1,C62-Supuestos!$C$32+1),0)-IF(C62&gt;$C$7,INDEX($C$65:$BJ$65,1,C62-$C$7),0))*Supuestos!$C$18</f>
@@ -16737,7 +16796,7 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1"/>
       <c r="B69" s="7" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C69" s="19" t="n">
         <f aca="false">C67-C68</f>
@@ -16983,7 +17042,7 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1"/>
       <c r="B70" s="7" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C70" s="19" t="n">
         <f aca="false">C64*$C$5</f>
@@ -17229,7 +17288,7 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1"/>
       <c r="B71" s="7" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C71" s="19" t="n">
         <f aca="false">C70</f>
@@ -17475,7 +17534,7 @@
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1"/>
       <c r="B72" s="7" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C72" s="19" t="n">
         <f aca="false">C71*$C$6</f>
@@ -17721,7 +17780,7 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1"/>
       <c r="B73" s="7" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C73" s="19" t="n">
         <f aca="false">C66*$C$8</f>
@@ -17967,7 +18026,7 @@
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1"/>
       <c r="B74" s="7" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C74" s="19" t="n">
         <f aca="false">MAX(0,MIN(C71,C73-C72))</f>
@@ -18213,7 +18272,7 @@
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1"/>
       <c r="B75" s="23" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C75" s="20" t="n">
         <f aca="false">C71-C74</f>
@@ -18459,7 +18518,7 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1"/>
       <c r="B76" s="7" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="C76" s="25" t="n">
         <f aca="false">C67*Supuestos!$C$11</f>
@@ -18705,7 +18764,7 @@
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1"/>
       <c r="B77" s="7" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C77" s="19" t="n">
         <f aca="false">IF(Supuestos!$C$19=0,0,C76/Supuestos!$C$19)</f>
@@ -18951,7 +19010,7 @@
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1"/>
       <c r="B78" s="7" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C78" s="19" t="n">
         <f aca="false">C67</f>
@@ -19197,253 +19256,253 @@
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1"/>
       <c r="B79" s="7" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,C78,C64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,C78,C64*Supuestos!$C$18)</f>
         <v>2</v>
       </c>
       <c r="D79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,D78-C78,D64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,D78-C78,D64*Supuestos!$C$18)</f>
         <v>3</v>
       </c>
       <c r="E79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,E78-D78,E64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,E78-D78,E64*Supuestos!$C$18)</f>
         <v>5</v>
       </c>
       <c r="F79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,F78-E78,F64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,F78-E78,F64*Supuestos!$C$18)</f>
         <v>6</v>
       </c>
       <c r="G79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,G78-F78,G64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,G78-F78,G64*Supuestos!$C$18)</f>
         <v>7</v>
       </c>
       <c r="H79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,H78-G78,H64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,H78-G78,H64*Supuestos!$C$18)</f>
         <v>8</v>
       </c>
       <c r="I79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,I78-H78,I64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,I78-H78,I64*Supuestos!$C$18)</f>
         <v>10</v>
       </c>
       <c r="J79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,J78-I78,J64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,J78-I78,J64*Supuestos!$C$18)</f>
         <v>11</v>
       </c>
       <c r="K79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,K78-J78,K64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,K78-J78,K64*Supuestos!$C$18)</f>
         <v>12</v>
       </c>
       <c r="L79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,L78-K78,L64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,L78-K78,L64*Supuestos!$C$18)</f>
         <v>13</v>
       </c>
       <c r="M79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,M78-L78,M64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,M78-L78,M64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="N79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,N78-M78,N64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,N78-M78,N64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="O79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,O78-N78,O64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,O78-N78,O64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="P79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,P78-O78,P64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,P78-O78,P64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="Q79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,Q78-P78,Q64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,Q78-P78,Q64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="R79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,R78-Q78,R64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,R78-Q78,R64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="S79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,S78-R78,S64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,S78-R78,S64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="T79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,T78-S78,T64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,T78-S78,T64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="U79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,U78-T78,U64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,U78-T78,U64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="V79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,V78-U78,V64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,V78-U78,V64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="W79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,W78-V78,W64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,W78-V78,W64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="X79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,X78-W78,X64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,X78-W78,X64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="Y79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,Y78-X78,Y64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,Y78-X78,Y64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="Z79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,Z78-Y78,Z64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,Z78-Y78,Z64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AA79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AA78-Z78,AA64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AA78-Z78,AA64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AB79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AB78-AA78,AB64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AB78-AA78,AB64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="AC79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AC78-AB78,AC64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AC78-AB78,AC64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AD79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AD78-AC78,AD64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AD78-AC78,AD64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AE79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AE78-AD78,AE64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AE78-AD78,AE64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="AF79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AF78-AE78,AF64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AF78-AE78,AF64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AG79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AG78-AF78,AG64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AG78-AF78,AG64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AH79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AH78-AG78,AH64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AH78-AG78,AH64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AI79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AI78-AH78,AI64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AI78-AH78,AI64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="AJ79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AJ78-AI78,AJ64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AJ78-AI78,AJ64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AK79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AK78-AJ78,AK64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AK78-AJ78,AK64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AL79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AL78-AK78,AL64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AL78-AK78,AL64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AM79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AM78-AL78,AM64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AM78-AL78,AM64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="AN79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AN78-AM78,AN64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AN78-AM78,AN64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AO79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AO78-AN78,AO64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AO78-AN78,AO64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AP79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AP78-AO78,AP64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AP78-AO78,AP64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AQ79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AQ78-AP78,AQ64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AQ78-AP78,AQ64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AR79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AR78-AQ78,AR64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AR78-AQ78,AR64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AS79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AS78-AR78,AS64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AS78-AR78,AS64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AT79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AT78-AS78,AT64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AT78-AS78,AT64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="AU79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AU78-AT78,AU64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AU78-AT78,AU64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AV79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AV78-AU78,AV64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AV78-AU78,AV64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AW79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AW78-AV78,AW64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AW78-AV78,AW64*Supuestos!$C$18)</f>
         <v>15</v>
       </c>
       <c r="AX79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AX78-AW78,AX64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AX78-AW78,AX64*Supuestos!$C$18)</f>
         <v>16</v>
       </c>
       <c r="AY79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AY78-AX78,AY64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AY78-AX78,AY64*Supuestos!$C$18)</f>
         <v>14</v>
       </c>
       <c r="AZ79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,AZ78-AY78,AZ64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,AZ78-AY78,AZ64*Supuestos!$C$18)</f>
         <v>13</v>
       </c>
       <c r="BA79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BA78-AZ78,BA64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BA78-AZ78,BA64*Supuestos!$C$18)</f>
         <v>12</v>
       </c>
       <c r="BB79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BB78-BA78,BB64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BB78-BA78,BB64*Supuestos!$C$18)</f>
         <v>11</v>
       </c>
       <c r="BC79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BC78-BB78,BC64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BC78-BB78,BC64*Supuestos!$C$18)</f>
         <v>9</v>
       </c>
       <c r="BD79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BD78-BC78,BD64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BD78-BC78,BD64*Supuestos!$C$18)</f>
         <v>8</v>
       </c>
       <c r="BE79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BE78-BD78,BE64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BE78-BD78,BE64*Supuestos!$C$18)</f>
         <v>7</v>
       </c>
       <c r="BF79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BF78-BE78,BF64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BF78-BE78,BF64*Supuestos!$C$18)</f>
         <v>5</v>
       </c>
       <c r="BG79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BG78-BF78,BG64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BG78-BF78,BG64*Supuestos!$C$18)</f>
         <v>4</v>
       </c>
       <c r="BH79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BH78-BG78,BH64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BH78-BG78,BH64*Supuestos!$C$18)</f>
         <v>3</v>
       </c>
       <c r="BI79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BI78-BH78,BI64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BI78-BH78,BI64*Supuestos!$C$18)</f>
         <v>2</v>
       </c>
       <c r="BJ79" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,BJ78-BI78,BJ64*Supuestos!$C$18)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,BJ78-BI78,BJ64*Supuestos!$C$18)</f>
         <v>0</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1"/>
       <c r="B80" s="7" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C80" s="44" t="n">
         <f aca="false">IF(C67&gt;=Supuestos!$C$43,C62,999)</f>
@@ -19777,7 +19836,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -19843,7 +19902,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -19973,7 +20032,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="23" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C5" s="45" t="n">
         <f aca="false">'Cartera 60M'!C62</f>
@@ -20219,7 +20278,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="7" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C6" s="25" t="n">
         <f aca="false">'Cartera 60M'!C63</f>
@@ -20465,7 +20524,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="7" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">'Cartera 60M'!C66</f>
@@ -20711,7 +20770,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="7" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C8" s="25" t="n">
         <f aca="false">'Cartera 60M'!C67</f>
@@ -20957,7 +21016,7 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="7" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">'Cartera 60M'!C75</f>
@@ -21267,7 +21326,7 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="6" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -21333,7 +21392,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="7" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">'Cartera 60M'!C70*Supuestos!$C$17</f>
@@ -21579,7 +21638,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="7" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C13" s="25" t="n">
         <f aca="false">'Cartera 60M'!C72</f>
@@ -21825,7 +21884,7 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="7" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">'Cartera 60M'!C76*Supuestos!$C$20*(1-Supuestos!$C$33)</f>
@@ -22071,7 +22130,7 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="23" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C15" s="22" t="n">
         <f aca="false">SUM(C12:C14)</f>
@@ -22381,7 +22440,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="6" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
@@ -22447,7 +22506,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="7" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">'Cartera 60M'!C71*Supuestos!$C$16/12</f>
@@ -22693,7 +22752,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="7" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C19" s="19" t="n">
         <f aca="false">'Cartera 60M'!C73*Supuestos!$C$34</f>
@@ -22939,7 +22998,7 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="7" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C20" s="19" t="n">
         <f aca="false">'Cartera 60M'!C68*Supuestos!$D$31+'Cartera 60M'!C69*Supuestos!$D$30</f>
@@ -23185,7 +23244,7 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="7" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">MAX(0,C30-C29)</f>
@@ -23431,7 +23490,7 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="7" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C22" s="19" t="n">
         <f aca="false">IF(C5=1,Supuestos!$D$40*Supuestos!$C$41,0)+IF(C5='Cartera 60M'!$C$18,Supuestos!$D$40*(1-Supuestos!$C$41),0)</f>
@@ -23677,7 +23736,7 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="23" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C23" s="22" t="n">
         <f aca="false">SUM(C18:C22)</f>
@@ -23987,7 +24046,7 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="23" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C25" s="20" t="n">
         <f aca="false">C15-C23</f>
@@ -24233,7 +24292,7 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
       <c r="B26" s="23" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C26" s="20" t="n">
         <f aca="false">C25</f>
@@ -24479,7 +24538,7 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="7" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">IF(C15=0,0,C25/C15)</f>
@@ -24725,7 +24784,7 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
       <c r="B28" s="6" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="15"/>
@@ -24791,7 +24850,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1"/>
       <c r="B29" s="7" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C29" s="19" t="n">
         <f aca="false">'Cartera 60M'!C76*Supuestos!$C$20*Supuestos!$C$33+C19+C20</f>
@@ -25037,7 +25096,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1"/>
       <c r="B30" s="7" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C30" s="19" t="n">
         <f aca="false">IF(C5&lt;=Supuestos!$C$36,Supuestos!$D$35,IF(C5&lt;=Supuestos!$C$38,Supuestos!$D$37,Supuestos!$D$39))</f>
@@ -25283,7 +25342,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1"/>
       <c r="B31" s="23" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C31" s="20" t="n">
         <f aca="false">MAX(C29,C30)+C22</f>
@@ -25529,7 +25588,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="7" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C32" s="44" t="n">
         <f aca="false">IF(C26&gt;=0,C5,999)</f>
@@ -25863,7 +25922,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -25929,7 +25988,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -26059,7 +26118,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="23" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C5" s="45" t="n">
         <f aca="false">'Cartera 60M'!C62</f>
@@ -26305,7 +26364,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="7" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C6" s="25" t="n">
         <f aca="false">'Cartera 60M'!C63</f>
@@ -26551,7 +26610,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="7" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">'Cartera 60M'!C66</f>
@@ -26797,7 +26856,7 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="7" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C8" s="25" t="n">
         <f aca="false">'Cartera 60M'!C67</f>
@@ -27043,7 +27102,7 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="7" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">'Cartera 60M'!C75</f>
@@ -27353,7 +27412,7 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="6" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -27419,7 +27478,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="7" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">'Cartera 60M'!C70*Supuestos!$C$17</f>
@@ -27665,7 +27724,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="7" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C13" s="25" t="n">
         <f aca="false">'Cartera 60M'!C72</f>
@@ -27911,253 +27970,253 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="7" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="C14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!C76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!C76*Supuestos!$C$59</f>
         <v>12000</v>
       </c>
       <c r="D14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!D76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!D76*Supuestos!$C$59</f>
         <v>30000</v>
       </c>
       <c r="E14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!E76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!E76*Supuestos!$C$59</f>
         <v>60000</v>
       </c>
       <c r="F14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!F76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!F76*Supuestos!$C$59</f>
         <v>96000</v>
       </c>
       <c r="G14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!G76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!G76*Supuestos!$C$59</f>
         <v>138000</v>
       </c>
       <c r="H14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!H76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!H76*Supuestos!$C$59</f>
         <v>186000</v>
       </c>
       <c r="I14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!I76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!I76*Supuestos!$C$59</f>
         <v>246000</v>
       </c>
       <c r="J14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!J76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!J76*Supuestos!$C$59</f>
         <v>312000</v>
       </c>
       <c r="K14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!K76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!K76*Supuestos!$C$59</f>
         <v>384000</v>
       </c>
       <c r="L14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!L76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!L76*Supuestos!$C$59</f>
         <v>462000</v>
       </c>
       <c r="M14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!M76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!M76*Supuestos!$C$59</f>
         <v>552000</v>
       </c>
       <c r="N14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!N76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!N76*Supuestos!$C$59</f>
         <v>648000</v>
       </c>
       <c r="O14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!O76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!O76*Supuestos!$C$59</f>
         <v>738000</v>
       </c>
       <c r="P14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!P76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!P76*Supuestos!$C$59</f>
         <v>828000</v>
       </c>
       <c r="Q14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!Q76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!Q76*Supuestos!$C$59</f>
         <v>918000</v>
       </c>
       <c r="R14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!R76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!R76*Supuestos!$C$59</f>
         <v>1008000</v>
       </c>
       <c r="S14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!S76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!S76*Supuestos!$C$59</f>
         <v>1098000</v>
       </c>
       <c r="T14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!T76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!T76*Supuestos!$C$59</f>
         <v>1194000</v>
       </c>
       <c r="U14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!U76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!U76*Supuestos!$C$59</f>
         <v>1284000</v>
       </c>
       <c r="V14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!V76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!V76*Supuestos!$C$59</f>
         <v>1374000</v>
       </c>
       <c r="W14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!W76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!W76*Supuestos!$C$59</f>
         <v>1464000</v>
       </c>
       <c r="X14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!X76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!X76*Supuestos!$C$59</f>
         <v>1560000</v>
       </c>
       <c r="Y14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!Y76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!Y76*Supuestos!$C$59</f>
         <v>1650000</v>
       </c>
       <c r="Z14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!Z76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!Z76*Supuestos!$C$59</f>
         <v>1740000</v>
       </c>
       <c r="AA14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AA76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AA76*Supuestos!$C$59</f>
         <v>1830000</v>
       </c>
       <c r="AB14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AB76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AB76*Supuestos!$C$59</f>
         <v>1926000</v>
       </c>
       <c r="AC14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AC76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AC76*Supuestos!$C$59</f>
         <v>2016000</v>
       </c>
       <c r="AD14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AD76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AD76*Supuestos!$C$59</f>
         <v>2106000</v>
       </c>
       <c r="AE14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AE76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AE76*Supuestos!$C$59</f>
         <v>2202000</v>
       </c>
       <c r="AF14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AF76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AF76*Supuestos!$C$59</f>
         <v>2292000</v>
       </c>
       <c r="AG14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AG76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AG76*Supuestos!$C$59</f>
         <v>2382000</v>
       </c>
       <c r="AH14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AH76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AH76*Supuestos!$C$59</f>
         <v>2472000</v>
       </c>
       <c r="AI14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AI76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AI76*Supuestos!$C$59</f>
         <v>2568000</v>
       </c>
       <c r="AJ14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AJ76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AJ76*Supuestos!$C$59</f>
         <v>2658000</v>
       </c>
       <c r="AK14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AK76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AK76*Supuestos!$C$59</f>
         <v>2748000</v>
       </c>
       <c r="AL14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AL76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AL76*Supuestos!$C$59</f>
         <v>2838000</v>
       </c>
       <c r="AM14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AM76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AM76*Supuestos!$C$59</f>
         <v>2934000</v>
       </c>
       <c r="AN14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AN76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AN76*Supuestos!$C$59</f>
         <v>3024000</v>
       </c>
       <c r="AO14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AO76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AO76*Supuestos!$C$59</f>
         <v>3114000</v>
       </c>
       <c r="AP14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AP76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AP76*Supuestos!$C$59</f>
         <v>3204000</v>
       </c>
       <c r="AQ14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AQ76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AQ76*Supuestos!$C$59</f>
         <v>3294000</v>
       </c>
       <c r="AR14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AR76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AR76*Supuestos!$C$59</f>
         <v>3384000</v>
       </c>
       <c r="AS14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AS76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AS76*Supuestos!$C$59</f>
         <v>3474000</v>
       </c>
       <c r="AT14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AT76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AT76*Supuestos!$C$59</f>
         <v>3570000</v>
       </c>
       <c r="AU14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AU76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AU76*Supuestos!$C$59</f>
         <v>3660000</v>
       </c>
       <c r="AV14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AV76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AV76*Supuestos!$C$59</f>
         <v>3750000</v>
       </c>
       <c r="AW14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AW76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AW76*Supuestos!$C$59</f>
         <v>3840000</v>
       </c>
       <c r="AX14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AX76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AX76*Supuestos!$C$59</f>
         <v>3936000</v>
       </c>
       <c r="AY14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AY76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AY76*Supuestos!$C$59</f>
         <v>4020000</v>
       </c>
       <c r="AZ14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AZ76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!AZ76*Supuestos!$C$59</f>
         <v>4098000</v>
       </c>
       <c r="BA14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BA76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BA76*Supuestos!$C$59</f>
         <v>4170000</v>
       </c>
       <c r="BB14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BB76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BB76*Supuestos!$C$59</f>
         <v>4236000</v>
       </c>
       <c r="BC14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BC76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BC76*Supuestos!$C$59</f>
         <v>4290000</v>
       </c>
       <c r="BD14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BD76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BD76*Supuestos!$C$59</f>
         <v>4338000</v>
       </c>
       <c r="BE14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BE76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BE76*Supuestos!$C$59</f>
         <v>4380000</v>
       </c>
       <c r="BF14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BF76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BF76*Supuestos!$C$59</f>
         <v>4410000</v>
       </c>
       <c r="BG14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BG76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BG76*Supuestos!$C$59</f>
         <v>4434000</v>
       </c>
       <c r="BH14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BH76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BH76*Supuestos!$C$59</f>
         <v>4452000</v>
       </c>
       <c r="BI14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BI76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BI76*Supuestos!$C$59</f>
         <v>4464000</v>
       </c>
       <c r="BJ14" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BJ76*Supuestos!$C$57</f>
+        <f aca="false">'Cartera 60M'!BJ76*Supuestos!$C$59</f>
         <v>4464000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="23" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C15" s="22" t="n">
         <f aca="false">SUM(C12:C14)</f>
@@ -28467,7 +28526,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="6" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
@@ -28533,7 +28592,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="7" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">'Cartera 60M'!C71*Supuestos!$C$16/12</f>
@@ -28779,7 +28838,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="7" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C19" s="25" t="n">
         <f aca="false">Supuestos!$D$50</f>
@@ -29025,499 +29084,499 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="7" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="C20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!C77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!C77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>2040</v>
       </c>
       <c r="D20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!D77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!D77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>5100</v>
       </c>
       <c r="E20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!E77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!E77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>10200</v>
       </c>
       <c r="F20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!F77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!F77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>16320</v>
       </c>
       <c r="G20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!G77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!G77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>23460</v>
       </c>
       <c r="H20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!H77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!H77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>31620</v>
       </c>
       <c r="I20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!I77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!I77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>41820</v>
       </c>
       <c r="J20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!J77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!J77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>53040</v>
       </c>
       <c r="K20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!K77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!K77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>65280</v>
       </c>
       <c r="L20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!L77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!L77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>78540</v>
       </c>
       <c r="M20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!M77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!M77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>93840</v>
       </c>
       <c r="N20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!N77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!N77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>110160</v>
       </c>
       <c r="O20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!O77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!O77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>125460</v>
       </c>
       <c r="P20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!P77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!P77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>140760</v>
       </c>
       <c r="Q20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!Q77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!Q77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>156060</v>
       </c>
       <c r="R20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!R77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!R77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>171360</v>
       </c>
       <c r="S20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!S77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!S77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>186660</v>
       </c>
       <c r="T20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!T77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!T77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>202980</v>
       </c>
       <c r="U20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!U77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!U77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>218280</v>
       </c>
       <c r="V20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!V77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!V77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>233580</v>
       </c>
       <c r="W20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!W77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!W77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>248880</v>
       </c>
       <c r="X20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!X77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!X77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>265200</v>
       </c>
       <c r="Y20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!Y77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!Y77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>280500</v>
       </c>
       <c r="Z20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!Z77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!Z77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>295800</v>
       </c>
       <c r="AA20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AA77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AA77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>311100</v>
       </c>
       <c r="AB20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AB77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AB77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>327420</v>
       </c>
       <c r="AC20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AC77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AC77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>342720</v>
       </c>
       <c r="AD20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AD77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AD77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>358020</v>
       </c>
       <c r="AE20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AE77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AE77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>374340</v>
       </c>
       <c r="AF20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AF77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AF77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>389640</v>
       </c>
       <c r="AG20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AG77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AG77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>404940</v>
       </c>
       <c r="AH20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AH77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AH77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>420240</v>
       </c>
       <c r="AI20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AI77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AI77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>436560</v>
       </c>
       <c r="AJ20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AJ77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AJ77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>451860</v>
       </c>
       <c r="AK20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AK77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AK77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>467160</v>
       </c>
       <c r="AL20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AL77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AL77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>482460</v>
       </c>
       <c r="AM20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AM77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AM77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>498780</v>
       </c>
       <c r="AN20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AN77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AN77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>514080</v>
       </c>
       <c r="AO20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AO77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AO77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>529380</v>
       </c>
       <c r="AP20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AP77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AP77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>544680</v>
       </c>
       <c r="AQ20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AQ77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AQ77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>559980</v>
       </c>
       <c r="AR20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AR77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AR77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>575280</v>
       </c>
       <c r="AS20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AS77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AS77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>590580</v>
       </c>
       <c r="AT20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AT77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AT77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>606900</v>
       </c>
       <c r="AU20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AU77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AU77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>622200</v>
       </c>
       <c r="AV20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AV77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AV77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>637500</v>
       </c>
       <c r="AW20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AW77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AW77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>652800</v>
       </c>
       <c r="AX20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AX77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AX77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>669120</v>
       </c>
       <c r="AY20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AY77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AY77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>683400</v>
       </c>
       <c r="AZ20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!AZ77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!AZ77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>696660</v>
       </c>
       <c r="BA20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BA77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BA77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>708900</v>
       </c>
       <c r="BB20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BB77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BB77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>720120</v>
       </c>
       <c r="BC20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BC77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BC77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>729300</v>
       </c>
       <c r="BD20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BD77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BD77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>737460</v>
       </c>
       <c r="BE20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BE77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BE77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>744600</v>
       </c>
       <c r="BF20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BF77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BF77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>749700</v>
       </c>
       <c r="BG20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BG77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BG77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>753780</v>
       </c>
       <c r="BH20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BH77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BH77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>756840</v>
       </c>
       <c r="BI20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BI77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BI77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>758880</v>
       </c>
       <c r="BJ20" s="19" t="n">
-        <f aca="false">MAX('Cartera 60M'!BJ77*Supuestos!$C$51,Supuestos!$C$52)*Supuestos!$C$7</f>
+        <f aca="false">MAX('Cartera 60M'!BJ77*((1-Supuestos!$C$53)*Supuestos!$C$51+Supuestos!$C$53*Supuestos!$C$52),Supuestos!$C$54)*Supuestos!$C$7</f>
         <v>758880</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="7" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C21" s="19" t="n">
-        <f aca="false">IF(AND(C5&gt;=Supuestos!$C$54,MOD(C5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(C5&gt;=Supuestos!$C$56,MOD(C5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="D21" s="19" t="n">
-        <f aca="false">IF(AND(D5&gt;=Supuestos!$C$54,MOD(D5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(D5&gt;=Supuestos!$C$56,MOD(D5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="E21" s="19" t="n">
-        <f aca="false">IF(AND(E5&gt;=Supuestos!$C$54,MOD(E5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(E5&gt;=Supuestos!$C$56,MOD(E5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="F21" s="19" t="n">
-        <f aca="false">IF(AND(F5&gt;=Supuestos!$C$54,MOD(F5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(F5&gt;=Supuestos!$C$56,MOD(F5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="G21" s="19" t="n">
-        <f aca="false">IF(AND(G5&gt;=Supuestos!$C$54,MOD(G5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(G5&gt;=Supuestos!$C$56,MOD(G5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="19" t="n">
-        <f aca="false">IF(AND(H5&gt;=Supuestos!$C$54,MOD(H5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(H5&gt;=Supuestos!$C$56,MOD(H5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="I21" s="19" t="n">
-        <f aca="false">IF(AND(I5&gt;=Supuestos!$C$54,MOD(I5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(I5&gt;=Supuestos!$C$56,MOD(I5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="19" t="n">
-        <f aca="false">IF(AND(J5&gt;=Supuestos!$C$54,MOD(J5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(J5&gt;=Supuestos!$C$56,MOD(J5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="K21" s="19" t="n">
-        <f aca="false">IF(AND(K5&gt;=Supuestos!$C$54,MOD(K5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(K5&gt;=Supuestos!$C$56,MOD(K5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="L21" s="19" t="n">
-        <f aca="false">IF(AND(L5&gt;=Supuestos!$C$54,MOD(L5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(L5&gt;=Supuestos!$C$56,MOD(L5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="M21" s="19" t="n">
-        <f aca="false">IF(AND(M5&gt;=Supuestos!$C$54,MOD(M5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(M5&gt;=Supuestos!$C$56,MOD(M5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="N21" s="19" t="n">
-        <f aca="false">IF(AND(N5&gt;=Supuestos!$C$54,MOD(N5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(N5&gt;=Supuestos!$C$56,MOD(N5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="O21" s="19" t="n">
-        <f aca="false">IF(AND(O5&gt;=Supuestos!$C$54,MOD(O5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(O5&gt;=Supuestos!$C$56,MOD(O5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>170000</v>
       </c>
       <c r="P21" s="19" t="n">
-        <f aca="false">IF(AND(P5&gt;=Supuestos!$C$54,MOD(P5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(P5&gt;=Supuestos!$C$56,MOD(P5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="Q21" s="19" t="n">
-        <f aca="false">IF(AND(Q5&gt;=Supuestos!$C$54,MOD(Q5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(Q5&gt;=Supuestos!$C$56,MOD(Q5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="R21" s="19" t="n">
-        <f aca="false">IF(AND(R5&gt;=Supuestos!$C$54,MOD(R5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(R5&gt;=Supuestos!$C$56,MOD(R5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="S21" s="19" t="n">
-        <f aca="false">IF(AND(S5&gt;=Supuestos!$C$54,MOD(S5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(S5&gt;=Supuestos!$C$56,MOD(S5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="T21" s="19" t="n">
-        <f aca="false">IF(AND(T5&gt;=Supuestos!$C$54,MOD(T5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(T5&gt;=Supuestos!$C$56,MOD(T5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="U21" s="19" t="n">
-        <f aca="false">IF(AND(U5&gt;=Supuestos!$C$54,MOD(U5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(U5&gt;=Supuestos!$C$56,MOD(U5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="V21" s="19" t="n">
-        <f aca="false">IF(AND(V5&gt;=Supuestos!$C$54,MOD(V5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(V5&gt;=Supuestos!$C$56,MOD(V5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="W21" s="19" t="n">
-        <f aca="false">IF(AND(W5&gt;=Supuestos!$C$54,MOD(W5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(W5&gt;=Supuestos!$C$56,MOD(W5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="X21" s="19" t="n">
-        <f aca="false">IF(AND(X5&gt;=Supuestos!$C$54,MOD(X5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(X5&gt;=Supuestos!$C$56,MOD(X5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="Y21" s="19" t="n">
-        <f aca="false">IF(AND(Y5&gt;=Supuestos!$C$54,MOD(Y5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(Y5&gt;=Supuestos!$C$56,MOD(Y5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="Z21" s="19" t="n">
-        <f aca="false">IF(AND(Z5&gt;=Supuestos!$C$54,MOD(Z5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(Z5&gt;=Supuestos!$C$56,MOD(Z5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AA21" s="19" t="n">
-        <f aca="false">IF(AND(AA5&gt;=Supuestos!$C$54,MOD(AA5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AA5&gt;=Supuestos!$C$56,MOD(AA5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>170000</v>
       </c>
       <c r="AB21" s="19" t="n">
-        <f aca="false">IF(AND(AB5&gt;=Supuestos!$C$54,MOD(AB5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AB5&gt;=Supuestos!$C$56,MOD(AB5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AC21" s="19" t="n">
-        <f aca="false">IF(AND(AC5&gt;=Supuestos!$C$54,MOD(AC5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AC5&gt;=Supuestos!$C$56,MOD(AC5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AD21" s="19" t="n">
-        <f aca="false">IF(AND(AD5&gt;=Supuestos!$C$54,MOD(AD5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AD5&gt;=Supuestos!$C$56,MOD(AD5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AE21" s="19" t="n">
-        <f aca="false">IF(AND(AE5&gt;=Supuestos!$C$54,MOD(AE5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AE5&gt;=Supuestos!$C$56,MOD(AE5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AF21" s="19" t="n">
-        <f aca="false">IF(AND(AF5&gt;=Supuestos!$C$54,MOD(AF5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AF5&gt;=Supuestos!$C$56,MOD(AF5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AG21" s="19" t="n">
-        <f aca="false">IF(AND(AG5&gt;=Supuestos!$C$54,MOD(AG5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AG5&gt;=Supuestos!$C$56,MOD(AG5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AH21" s="19" t="n">
-        <f aca="false">IF(AND(AH5&gt;=Supuestos!$C$54,MOD(AH5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AH5&gt;=Supuestos!$C$56,MOD(AH5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AI21" s="19" t="n">
-        <f aca="false">IF(AND(AI5&gt;=Supuestos!$C$54,MOD(AI5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AI5&gt;=Supuestos!$C$56,MOD(AI5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AJ21" s="19" t="n">
-        <f aca="false">IF(AND(AJ5&gt;=Supuestos!$C$54,MOD(AJ5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AJ5&gt;=Supuestos!$C$56,MOD(AJ5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AK21" s="19" t="n">
-        <f aca="false">IF(AND(AK5&gt;=Supuestos!$C$54,MOD(AK5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AK5&gt;=Supuestos!$C$56,MOD(AK5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AL21" s="19" t="n">
-        <f aca="false">IF(AND(AL5&gt;=Supuestos!$C$54,MOD(AL5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AL5&gt;=Supuestos!$C$56,MOD(AL5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AM21" s="19" t="n">
-        <f aca="false">IF(AND(AM5&gt;=Supuestos!$C$54,MOD(AM5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AM5&gt;=Supuestos!$C$56,MOD(AM5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>170000</v>
       </c>
       <c r="AN21" s="19" t="n">
-        <f aca="false">IF(AND(AN5&gt;=Supuestos!$C$54,MOD(AN5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AN5&gt;=Supuestos!$C$56,MOD(AN5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AO21" s="19" t="n">
-        <f aca="false">IF(AND(AO5&gt;=Supuestos!$C$54,MOD(AO5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AO5&gt;=Supuestos!$C$56,MOD(AO5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AP21" s="19" t="n">
-        <f aca="false">IF(AND(AP5&gt;=Supuestos!$C$54,MOD(AP5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AP5&gt;=Supuestos!$C$56,MOD(AP5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AQ21" s="19" t="n">
-        <f aca="false">IF(AND(AQ5&gt;=Supuestos!$C$54,MOD(AQ5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AQ5&gt;=Supuestos!$C$56,MOD(AQ5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AR21" s="19" t="n">
-        <f aca="false">IF(AND(AR5&gt;=Supuestos!$C$54,MOD(AR5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AR5&gt;=Supuestos!$C$56,MOD(AR5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AS21" s="19" t="n">
-        <f aca="false">IF(AND(AS5&gt;=Supuestos!$C$54,MOD(AS5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AS5&gt;=Supuestos!$C$56,MOD(AS5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AT21" s="19" t="n">
-        <f aca="false">IF(AND(AT5&gt;=Supuestos!$C$54,MOD(AT5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AT5&gt;=Supuestos!$C$56,MOD(AT5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AU21" s="19" t="n">
-        <f aca="false">IF(AND(AU5&gt;=Supuestos!$C$54,MOD(AU5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AU5&gt;=Supuestos!$C$56,MOD(AU5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AV21" s="19" t="n">
-        <f aca="false">IF(AND(AV5&gt;=Supuestos!$C$54,MOD(AV5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AV5&gt;=Supuestos!$C$56,MOD(AV5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AW21" s="19" t="n">
-        <f aca="false">IF(AND(AW5&gt;=Supuestos!$C$54,MOD(AW5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AW5&gt;=Supuestos!$C$56,MOD(AW5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AX21" s="19" t="n">
-        <f aca="false">IF(AND(AX5&gt;=Supuestos!$C$54,MOD(AX5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AX5&gt;=Supuestos!$C$56,MOD(AX5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="AY21" s="19" t="n">
-        <f aca="false">IF(AND(AY5&gt;=Supuestos!$C$54,MOD(AY5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AY5&gt;=Supuestos!$C$56,MOD(AY5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>170000</v>
       </c>
       <c r="AZ21" s="19" t="n">
-        <f aca="false">IF(AND(AZ5&gt;=Supuestos!$C$54,MOD(AZ5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(AZ5&gt;=Supuestos!$C$56,MOD(AZ5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BA21" s="19" t="n">
-        <f aca="false">IF(AND(BA5&gt;=Supuestos!$C$54,MOD(BA5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BA5&gt;=Supuestos!$C$56,MOD(BA5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BB21" s="19" t="n">
-        <f aca="false">IF(AND(BB5&gt;=Supuestos!$C$54,MOD(BB5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BB5&gt;=Supuestos!$C$56,MOD(BB5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BC21" s="19" t="n">
-        <f aca="false">IF(AND(BC5&gt;=Supuestos!$C$54,MOD(BC5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BC5&gt;=Supuestos!$C$56,MOD(BC5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BD21" s="19" t="n">
-        <f aca="false">IF(AND(BD5&gt;=Supuestos!$C$54,MOD(BD5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BD5&gt;=Supuestos!$C$56,MOD(BD5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BE21" s="19" t="n">
-        <f aca="false">IF(AND(BE5&gt;=Supuestos!$C$54,MOD(BE5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BE5&gt;=Supuestos!$C$56,MOD(BE5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BF21" s="19" t="n">
-        <f aca="false">IF(AND(BF5&gt;=Supuestos!$C$54,MOD(BF5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BF5&gt;=Supuestos!$C$56,MOD(BF5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BG21" s="19" t="n">
-        <f aca="false">IF(AND(BG5&gt;=Supuestos!$C$54,MOD(BG5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BG5&gt;=Supuestos!$C$56,MOD(BG5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BH21" s="19" t="n">
-        <f aca="false">IF(AND(BH5&gt;=Supuestos!$C$54,MOD(BH5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BH5&gt;=Supuestos!$C$56,MOD(BH5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BI21" s="19" t="n">
-        <f aca="false">IF(AND(BI5&gt;=Supuestos!$C$54,MOD(BI5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BI5&gt;=Supuestos!$C$56,MOD(BI5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
       <c r="BJ21" s="19" t="n">
-        <f aca="false">IF(AND(BJ5&gt;=Supuestos!$C$54,MOD(BJ5-Supuestos!$C$54,12)=0),Supuestos!$D$53,0)</f>
+        <f aca="false">IF(AND(BJ5&gt;=Supuestos!$C$56,MOD(BJ5-Supuestos!$C$56,12)=0),Supuestos!$D$55,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="7" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C22" s="19" t="n">
         <f aca="false">IF(C5=1,Supuestos!$D$46,0)</f>
@@ -29763,499 +29822,499 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="7" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!C79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!C79*Supuestos!$D$57</f>
         <v>4454</v>
       </c>
       <c r="D23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!D79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!D79*Supuestos!$D$57</f>
         <v>6681</v>
       </c>
       <c r="E23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!E79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!E79*Supuestos!$D$57</f>
         <v>11135</v>
       </c>
       <c r="F23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!F79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!F79*Supuestos!$D$57</f>
         <v>13362</v>
       </c>
       <c r="G23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!G79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!G79*Supuestos!$D$57</f>
         <v>15589</v>
       </c>
       <c r="H23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!H79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!H79*Supuestos!$D$57</f>
         <v>17816</v>
       </c>
       <c r="I23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!I79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!I79*Supuestos!$D$57</f>
         <v>22270</v>
       </c>
       <c r="J23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!J79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!J79*Supuestos!$D$57</f>
         <v>24497</v>
       </c>
       <c r="K23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!K79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!K79*Supuestos!$D$57</f>
         <v>26724</v>
       </c>
       <c r="L23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!L79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!L79*Supuestos!$D$57</f>
         <v>28951</v>
       </c>
       <c r="M23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!M79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!M79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="N23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!N79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!N79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="O23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!O79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!O79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="P23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!P79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!P79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="Q23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!Q79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!Q79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="R23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!R79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!R79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="S23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!S79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!S79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="T23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!T79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!T79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="U23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!U79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!U79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="V23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!V79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!V79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="W23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!W79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!W79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="X23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!X79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!X79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="Y23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!Y79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!Y79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="Z23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!Z79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!Z79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AA23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AA79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AA79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AB23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AB79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AB79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="AC23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AC79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AC79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AD23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AD79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AD79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AE23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AE79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AE79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="AF23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AF79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AF79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AG23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AG79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AG79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AH23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AH79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AH79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AI23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AI79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AI79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="AJ23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AJ79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AJ79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AK23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AK79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AK79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AL23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AL79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AL79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AM23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AM79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AM79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="AN23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AN79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AN79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AO23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AO79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AO79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AP23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AP79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AP79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AQ23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AQ79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AQ79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AR23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AR79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AR79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AS23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AS79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AS79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AT23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AT79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AT79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="AU23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AU79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AU79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AV23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AV79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AV79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AW23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AW79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AW79*Supuestos!$D$57</f>
         <v>33405</v>
       </c>
       <c r="AX23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AX79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AX79*Supuestos!$D$57</f>
         <v>35632</v>
       </c>
       <c r="AY23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AY79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AY79*Supuestos!$D$57</f>
         <v>31178</v>
       </c>
       <c r="AZ23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!AZ79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!AZ79*Supuestos!$D$57</f>
         <v>28951</v>
       </c>
       <c r="BA23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BA79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BA79*Supuestos!$D$57</f>
         <v>26724</v>
       </c>
       <c r="BB23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BB79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BB79*Supuestos!$D$57</f>
         <v>24497</v>
       </c>
       <c r="BC23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BC79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BC79*Supuestos!$D$57</f>
         <v>20043</v>
       </c>
       <c r="BD23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BD79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BD79*Supuestos!$D$57</f>
         <v>17816</v>
       </c>
       <c r="BE23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BE79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BE79*Supuestos!$D$57</f>
         <v>15589</v>
       </c>
       <c r="BF23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BF79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BF79*Supuestos!$D$57</f>
         <v>11135</v>
       </c>
       <c r="BG23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BG79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BG79*Supuestos!$D$57</f>
         <v>8908</v>
       </c>
       <c r="BH23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BH79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BH79*Supuestos!$D$57</f>
         <v>6681</v>
       </c>
       <c r="BI23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BI79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BI79*Supuestos!$D$57</f>
         <v>4454</v>
       </c>
       <c r="BJ23" s="19" t="n">
-        <f aca="false">'Cartera 60M'!BJ79*Supuestos!$D$55</f>
+        <f aca="false">'Cartera 60M'!BJ79*Supuestos!$D$57</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="7" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="D24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="E24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="F24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="G24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="H24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="I24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="J24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="K24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="L24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="M24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="N24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="O24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="P24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="Q24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="R24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="S24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="T24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="U24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="V24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="W24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="X24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="Y24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="Z24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AA24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AB24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AC24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AD24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AE24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AF24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AG24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AH24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AI24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AJ24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AK24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AL24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AM24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AN24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AO24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AP24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AQ24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AR24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AS24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AT24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AU24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AV24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AW24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AX24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AY24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="AZ24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BA24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BB24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BC24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BD24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BE24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BF24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BG24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BH24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BI24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
       <c r="BJ24" s="25" t="n">
-        <f aca="false">Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$C$60</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="23" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C25" s="22" t="n">
         <f aca="false">SUM(C18:C24)</f>
@@ -30565,7 +30624,7 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="23" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C27" s="20" t="n">
         <f aca="false">C15-C25</f>
@@ -30811,7 +30870,7 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
       <c r="B28" s="23" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">C27</f>
@@ -31057,7 +31116,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1"/>
       <c r="B29" s="7" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C29" s="12" t="n">
         <f aca="false">IF(C15=0,0,C27/C15)</f>
@@ -31303,7 +31362,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1"/>
       <c r="B30" s="6" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
@@ -31369,7 +31428,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1"/>
       <c r="B31" s="23" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C31" s="20" t="n">
         <f aca="false">SUM(C19:C23)</f>
@@ -31615,7 +31674,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="7" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C32" s="44" t="n">
         <f aca="false">IF(C28&gt;=0,C5,999)</f>
@@ -31894,7 +31953,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -31904,7 +31963,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -31922,7 +31981,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>4</v>
@@ -31936,7 +31995,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="7" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C6" s="19" t="n">
         <f aca="false">Supuestos!$C$13*'Cartera 60M'!$C$12/Supuestos!$C$15</f>
@@ -31952,7 +32011,7 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="7" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">C6*Supuestos!$C$14/12</f>
@@ -31968,14 +32027,14 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
       <c r="B8" s="7" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">Supuestos!$C$11*Supuestos!$C$20*(1-Supuestos!$C$33)*Supuestos!$C$18</f>
         <v>3000</v>
       </c>
       <c r="D8" s="19" t="n">
-        <f aca="false">Supuestos!$C$11*Supuestos!$C$57*Supuestos!$C$18</f>
+        <f aca="false">Supuestos!$C$11*Supuestos!$C$59*Supuestos!$C$18</f>
         <v>6000</v>
       </c>
       <c r="E8" s="1"/>
@@ -31984,7 +32043,7 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="7" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C9" s="19" t="n">
         <f aca="false">Supuestos!$C$13*Supuestos!$C$17/Supuestos!$C$15</f>
@@ -32000,7 +32059,7 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="23" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="C10" s="20" t="n">
         <f aca="false">SUM(C7:C9)</f>
@@ -32024,7 +32083,7 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">C6*Supuestos!$C$16/12</f>
@@ -32040,7 +32099,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="7" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="C13" s="19" t="n">
         <f aca="false">'Cartera 60M'!$C$8*Supuestos!$C$34</f>
@@ -32055,14 +32114,14 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="7" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">Supuestos!$D$31*Supuestos!$C$18</f>
         <v>255</v>
       </c>
       <c r="D14" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$19=0,0,Supuestos!$C$11/Supuestos!$C$19)*Supuestos!$D$51*Supuestos!$C$18</f>
+        <f aca="false">IF(Supuestos!$C$19=0,0,Supuestos!$C$11/Supuestos!$C$19)*((1-Supuestos!$C$53)*Supuestos!$D$51+Supuestos!$C$53*Supuestos!$D$52)*Supuestos!$C$18</f>
         <v>1020</v>
       </c>
       <c r="E14" s="1"/>
@@ -32071,13 +32130,13 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="7" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="C15" s="19" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="19" t="n">
-        <f aca="false">IF(Supuestos!$C$56=1,0,Supuestos!$D$55*Supuestos!$C$18/Supuestos!$C$15)</f>
+        <f aca="false">IF(Supuestos!$C$58=1,0,Supuestos!$D$57*Supuestos!$C$18/Supuestos!$C$15)</f>
         <v>0</v>
       </c>
       <c r="E15" s="1"/>
@@ -32086,7 +32145,7 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
       <c r="B16" s="23" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C16" s="20" t="n">
         <f aca="false">SUM(C12:C15)</f>
@@ -32102,7 +32161,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="23" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="C17" s="20" t="n">
         <f aca="false">C10-C16</f>
@@ -32126,14 +32185,14 @@
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="46" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="C19" s="25" t="n">
         <f aca="false">Supuestos!$D$39</f>
         <v>85000</v>
       </c>
       <c r="D19" s="19" t="n">
-        <f aca="false">Supuestos!$D$50+Supuestos!$D$53/12+Supuestos!$C$58</f>
+        <f aca="false">Supuestos!$D$50+Supuestos!$D$55/12+Supuestos!$C$60</f>
         <v>81316.6666666667</v>
       </c>
       <c r="E19" s="1"/>
@@ -32142,7 +32201,7 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="7" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C20" s="19" t="n">
         <f aca="false">Supuestos!$C$11*Supuestos!$C$20*Supuestos!$C$33*Supuestos!$C$18+C13+C14</f>
@@ -32165,7 +32224,7 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="23" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="C22" s="20" t="n">
         <f aca="false">IF(C17&lt;=0,"no se alcanza",ROUNDUP(C19/(C17+C20),0))</f>
@@ -32189,14 +32248,14 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C24" s="24" t="n">
         <f aca="false">IF(D17&lt;=C17,"nunca",IF(C20&lt;=0,ROUNDUP(MAX(0,D19-C19)/(D17-C17),0),IF((C19/C20)*(D17-C17)-D19&lt;0,ROUNDUP(D19/(D17-C17),0),IF(C19-D19&gt;=0,0,ROUNDUP((D19-C19)/(D17-C17-C20),0)))))</f>
         <v>25</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -32212,7 +32271,7 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
       <c r="B26" s="6" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
@@ -32222,7 +32281,7 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="16" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>4</v>
@@ -32231,10 +32290,10 @@
         <v>5</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32534,7 +32593,7 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1"/>
       <c r="B42" s="3" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>

</xml_diff>